<commit_message>
feat: teach ledger_qa two checks the article series surfaced
1. Material-vs-year cross check: a PVC-family pipe whose construction year
   predates JSWAS K-1 (1974) is flagged (catches the 1955 PVC record found
   while writing the generation-shift article).
2. Scoped business-key uniqueness: report blank keys, raw duplicates, AND
   within-system duplicates separately. Handa's manhole keys are unique only
   per drainage system (2,505 cross-system reuses vs 2 real duplicates), so
   a raw count alone misleads the remediation estimate.
</commit_message>
<xml_diff>
--- a/work1-ledger-cleanup/qa_report.xlsx
+++ b/work1-ledger-cleanup/qa_report.xlsx
@@ -463,7 +463,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="4">
@@ -473,7 +473,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5">
@@ -483,7 +483,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6">
@@ -509,14 +509,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E99"/>
+  <dimension ref="A1:E103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="7" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2095,20 +2095,20 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>土被りの欠損(SAFIELD003)</t>
+          <t>管種×年代の整合(塩ビ系)</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>NG</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>1660</v>
+        <v>1</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>欠損率 7.8%</t>
+          <t>JSWAS K-1 制定(1974)より前の施工年度。桁誤り・管種誤記・更生の未反映等の疑い</t>
         </is>
       </c>
     </row>
@@ -2120,20 +2120,20 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>土被り異常値(SAFIELD003)</t>
+          <t>土被りの欠損(SAFIELD003)</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>NG</t>
+          <t>要確認</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>141</v>
+        <v>1660</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>許容 0.0-15.0m。負値・桁違いを検出</t>
+          <t>欠損率 7.8%</t>
         </is>
       </c>
     </row>
@@ -2145,20 +2145,20 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>土被りの欠損(SAFIELD004)</t>
+          <t>土被り異常値(SAFIELD003)</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>NG</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>2027</v>
+        <v>141</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>欠損率 9.6%</t>
+          <t>許容 0.0-15.0m。負値・桁違いを検出</t>
         </is>
       </c>
     </row>
@@ -2170,32 +2170,32 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>土被り異常値(SAFIELD004)</t>
+          <t>土被りの欠損(SAFIELD004)</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>NG</t>
+          <t>要確認</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>189</v>
+        <v>2027</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>許容 0.0-15.0m。負値・桁違いを検出</t>
+          <t>欠損率 9.6%</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>下水_マンホール</t>
+          <t>下水_管渠</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>座標系定義(.prj)</t>
+          <t>土被り異常値(SAFIELD004)</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -2204,11 +2204,11 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>1</v>
+        <v>189</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>空または欠落。座標範囲からの推定と検証が必要</t>
+          <t>許容 0.0-15.0m。負値・桁違いを検出</t>
         </is>
       </c>
     </row>
@@ -2220,18 +2220,22 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>属性定義XML</t>
+          <t>座標系定義(.prj)</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>NG</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>0</v>
-      </c>
-      <c r="E72" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>空または欠落。座標範囲からの推定と検証が必要</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -2241,16 +2245,16 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>レコード数</t>
+          <t>属性定義XML</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>20689</v>
+        <v>0</v>
       </c>
       <c r="E73" t="inlineStr"/>
     </row>
@@ -2262,16 +2266,16 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>空ジオメトリ</t>
+          <t>レコード数</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>0</v>
+        <v>20689</v>
       </c>
       <c r="E74" t="inlineStr"/>
     </row>
@@ -2283,16 +2287,16 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>SAUID重複</t>
+          <t>空ジオメトリ</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>NG</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E75" t="inlineStr"/>
     </row>
@@ -2304,22 +2308,18 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>表示様式(SASTYLEID)の混在</t>
+          <t>SAUID重複</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>NG</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>31</v>
-      </c>
-      <c r="E76" t="inlineStr">
-        <is>
-          <t>複数様式が1ファイルに混在。分析前に分類が必要</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="E76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -2329,7 +2329,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>年度の欠損</t>
+          <t>表示様式(SASTYLEID)の混在</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -2338,11 +2338,11 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>2616</v>
+        <v>31</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>欠損率 12.6%</t>
+          <t>複数様式が1ファイルに混在。分析前に分類が必要</t>
         </is>
       </c>
     </row>
@@ -2354,110 +2354,122 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>年度の範囲外</t>
+          <t>年度の欠損</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>要確認</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>0</v>
+        <v>2616</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>1900年未満または未来(暦年基準)</t>
+          <t>欠損率 12.6%</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>下水_取付管</t>
+          <t>下水_マンホール</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>座標系定義(.prj)</t>
+          <t>年度の範囲外</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>NG</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>空または欠落。座標範囲からの推定と検証が必要</t>
+          <t>1900年未満または未来(暦年基準)</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>下水_取付管</t>
+          <t>下水_マンホール</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>属性定義XML</t>
+          <t>人孔キーの欠損</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>NG</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>0</v>
-      </c>
-      <c r="E80" t="inlineStr"/>
+        <v>1726</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>施設を特定するキーが空</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>下水_取付管</t>
+          <t>下水_マンホール</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>レコード数</t>
+          <t>人孔キーの重複(系統内)</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>NG</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>39443</v>
-      </c>
-      <c r="E81" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>全体重複 2507 のうち系統内の真の重複は 2。残りは系統別採番(キーは系統内でのみ一意)によるもの</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>下水_取付管</t>
+          <t>下水_マンホール</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>空ジオメトリ</t>
+          <t>人孔キーの重複(全体)</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>要確認</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>0</v>
-      </c>
-      <c r="E82" t="inlineStr"/>
+        <v>2507</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>系統をまたぐ再利用を含む</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -2467,7 +2479,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>延長ほぼゼロの線</t>
+          <t>座標系定義(.prj)</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -2480,7 +2492,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>0.01(座標単位)未満。CRS未定義時は単位に注意</t>
+          <t>空または欠落。座標範囲からの推定と検証が必要</t>
         </is>
       </c>
     </row>
@@ -2492,16 +2504,16 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>SAUID重複</t>
+          <t>属性定義XML</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>NG</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="E84" t="inlineStr"/>
     </row>
@@ -2513,22 +2525,18 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>表示様式(SASTYLEID)の混在</t>
+          <t>レコード数</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>2</v>
-      </c>
-      <c r="E85" t="inlineStr">
-        <is>
-          <t>複数様式が1ファイルに混在。分析前に分類が必要</t>
-        </is>
-      </c>
+        <v>39443</v>
+      </c>
+      <c r="E85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -2538,7 +2546,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>口径の欠損</t>
+          <t>空ジオメトリ</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -2547,13 +2555,9 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>1392</v>
-      </c>
-      <c r="E86" t="inlineStr">
-        <is>
-          <t>欠損率 3.5%</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="E86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -2563,20 +2567,20 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>口径の未入力(0)</t>
+          <t>延長ほぼゼロの線</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>NG</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>0 は未入力プレースホルダとみなす</t>
+          <t>0.01(座標単位)未満。CRS未定義時は単位に注意</t>
         </is>
       </c>
     </row>
@@ -2588,22 +2592,18 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>口径の上限超過</t>
+          <t>SAUID重複</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>NG</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>179</v>
-      </c>
-      <c r="E88" t="inlineStr">
-        <is>
-          <t>300mm 超。大型構造物の実在可能性あり、現地資料と照合</t>
-        </is>
-      </c>
+        <v>96</v>
+      </c>
+      <c r="E88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -2613,57 +2613,57 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>口径の下限未満(入力疑義)</t>
+          <t>表示様式(SASTYLEID)の混在</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>NG</t>
+          <t>要確認</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>50mm 未満(0 を除く)。桁誤り等の疑い</t>
+          <t>複数様式が1ファイルに混在。分析前に分類が必要</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>下水_桝</t>
+          <t>下水_取付管</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>座標系定義(.prj)</t>
+          <t>口径の欠損</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>NG</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>1</v>
+        <v>1392</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>空または欠落。座標範囲からの推定と検証が必要</t>
+          <t>欠損率 3.5%</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>下水_桝</t>
+          <t>下水_取付管</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>属性定義XML</t>
+          <t>口径の未入力(0)</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -2674,49 +2674,61 @@
       <c r="D91" t="n">
         <v>0</v>
       </c>
-      <c r="E91" t="inlineStr"/>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>0 は未入力プレースホルダとみなす</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>下水_桝</t>
+          <t>下水_取付管</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>レコード数</t>
+          <t>口径の上限超過</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>要確認</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>39391</v>
-      </c>
-      <c r="E92" t="inlineStr"/>
+        <v>179</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>300mm 超。大型構造物の実在可能性あり、現地資料と照合</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>下水_桝</t>
+          <t>下水_取付管</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>空ジオメトリ</t>
+          <t>口径の下限未満(入力疑義)</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>NG</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>0</v>
-      </c>
-      <c r="E93" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>50mm 未満(0 を除く)。桁誤り等の疑い</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -2726,7 +2738,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>SAUID重複</t>
+          <t>座標系定義(.prj)</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -2735,9 +2747,13 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>66</v>
-      </c>
-      <c r="E94" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>空または欠落。座標範囲からの推定と検証が必要</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -2747,22 +2763,18 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>表示様式(SASTYLEID)の混在</t>
+          <t>属性定義XML</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>12</v>
-      </c>
-      <c r="E95" t="inlineStr">
-        <is>
-          <t>複数様式が1ファイルに混在。分析前に分類が必要</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="E95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -2772,22 +2784,18 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>口径の欠損</t>
+          <t>レコード数</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>1</v>
-      </c>
-      <c r="E96" t="inlineStr">
-        <is>
-          <t>欠損率 0.0%</t>
-        </is>
-      </c>
+        <v>39391</v>
+      </c>
+      <c r="E96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -2797,22 +2805,18 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>口径の未入力(0)</t>
+          <t>空ジオメトリ</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>2252</v>
-      </c>
-      <c r="E97" t="inlineStr">
-        <is>
-          <t>0 は未入力プレースホルダとみなす</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="E97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -2822,22 +2826,18 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>口径の上限超過</t>
+          <t>SAUID重複</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>要確認</t>
+          <t>NG</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>178</v>
-      </c>
-      <c r="E98" t="inlineStr">
-        <is>
-          <t>300mm 超。大型構造物の実在可能性あり、現地資料と照合</t>
-        </is>
-      </c>
+        <v>66</v>
+      </c>
+      <c r="E98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -2847,18 +2847,118 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
+          <t>表示様式(SASTYLEID)の混在</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>12</v>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>複数様式が1ファイルに混在。分析前に分類が必要</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>下水_桝</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>口径の欠損</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>1</v>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>欠損率 0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>下水_桝</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>口径の未入力(0)</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>2252</v>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>0 は未入力プレースホルダとみなす</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>下水_桝</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>口径の上限超過</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>178</v>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>300mm 超。大型構造物の実在可能性あり、現地資料と照合</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>下水_桝</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
           <t>口径の下限未満(入力疑義)</t>
         </is>
       </c>
-      <c r="C99" t="inlineStr">
-        <is>
-          <t>NG</t>
-        </is>
-      </c>
-      <c r="D99" t="n">
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>NG</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
         <v>3</v>
       </c>
-      <c r="E99" t="inlineStr">
+      <c r="E103" t="inlineStr">
         <is>
           <t>50mm 未満(0 を除く)。桁誤り等の疑い</t>
         </is>
@@ -2875,14 +2975,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="6" customWidth="1" min="3" max="3"/>
-    <col width="7" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3162,7 +3262,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>土被り異常値(SAFIELD003)</t>
+          <t>管種×年代の整合(塩ビ系)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -3171,11 +3271,11 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>141</v>
+        <v>1</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>許容 0.0-15.0m。負値・桁違いを検出</t>
+          <t>JSWAS K-1 制定(1974)より前の施工年度。桁誤り・管種誤記・更生の未反映等の疑い</t>
         </is>
       </c>
     </row>
@@ -3187,7 +3287,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>土被り異常値(SAFIELD004)</t>
+          <t>土被り異常値(SAFIELD003)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -3196,7 +3296,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>189</v>
+        <v>141</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -3207,12 +3307,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>下水_マンホール</t>
+          <t>下水_管渠</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>座標系定義(.prj)</t>
+          <t>土被り異常値(SAFIELD004)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -3221,11 +3321,11 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>1</v>
+        <v>189</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>空または欠落。座標範囲からの推定と検証が必要</t>
+          <t>許容 0.0-15.0m。負値・桁違いを検出</t>
         </is>
       </c>
     </row>
@@ -3237,7 +3337,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>SAUID重複</t>
+          <t>座標系定義(.prj)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -3246,19 +3346,23 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>2</v>
-      </c>
-      <c r="E15" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>空または欠落。座標範囲からの推定と検証が必要</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>下水_取付管</t>
+          <t>下水_マンホール</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>座標系定義(.prj)</t>
+          <t>SAUID重複</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -3267,23 +3371,19 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>1</v>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>空または欠落。座標範囲からの推定と検証が必要</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="E16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>下水_取付管</t>
+          <t>下水_マンホール</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>延長ほぼゼロの線</t>
+          <t>人孔キーの欠損</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -3292,23 +3392,23 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>1</v>
+        <v>1726</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>0.01(座標単位)未満。CRS未定義時は単位に注意</t>
+          <t>施設を特定するキーが空</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>下水_取付管</t>
+          <t>下水_マンホール</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>SAUID重複</t>
+          <t>人孔キーの重複(系統内)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -3317,9 +3417,13 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>96</v>
-      </c>
-      <c r="E18" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>全体重複 2507 のうち系統内の真の重複は 2。残りは系統別採番(キーは系統内でのみ一意)によるもの</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3329,7 +3433,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>口径の下限未満(入力疑義)</t>
+          <t>座標系定義(.prj)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -3338,23 +3442,23 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>50mm 未満(0 を除く)。桁誤り等の疑い</t>
+          <t>空または欠落。座標範囲からの推定と検証が必要</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>下水_桝</t>
+          <t>下水_取付管</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>座標系定義(.prj)</t>
+          <t>延長ほぼゼロの線</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -3367,14 +3471,14 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>空または欠落。座標範囲からの推定と検証が必要</t>
+          <t>0.01(座標単位)未満。CRS未定義時は単位に注意</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>下水_桝</t>
+          <t>下水_取付管</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -3388,14 +3492,14 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>66</v>
+        <v>96</v>
       </c>
       <c r="E21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>下水_桝</t>
+          <t>下水_取付管</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -3412,6 +3516,77 @@
         <v>3</v>
       </c>
       <c r="E22" t="inlineStr">
+        <is>
+          <t>50mm 未満(0 を除く)。桁誤り等の疑い</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>下水_桝</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>座標系定義(.prj)</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>NG</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>空または欠落。座標範囲からの推定と検証が必要</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>下水_桝</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>SAUID重複</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>NG</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>66</v>
+      </c>
+      <c r="E24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>下水_桝</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>口径の下限未満(入力疑義)</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>NG</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E25" t="inlineStr">
         <is>
           <t>50mm 未満(0 を除く)。桁誤り等の疑い</t>
         </is>

</xml_diff>